<commit_message>
Workbook: SUMIFS quarter-index windows (no OFFSET), live bridge formulas, no label clobber; single run_all entrypoint
The 4-quarter cell was keyed to row position (newest-first) and dropped the
selected quarter — a reviewer opening the workbook saw 534.2 where the README
promised 543.4. Windows now key to a Seq column (SUMIFS, sort-safe, blank
instead of #REF at the edges); the caveat moved off the metric label row; the
Annual bridge sheet computes write-offs, average rollover and both bridge
terms as live formulas. build_workbook.py scans every sheet for OFFSET (zero
found) and asserts the 4-quarter formula's row window sums to the Python value
(543.4 for the default selection on this pull). src/run_all.py runs the five
stages in order.
</commit_message>
<xml_diff>
--- a/outputs/quick_check.xlsx
+++ b/outputs/quick_check.xlsx
@@ -18,10 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0&quot;%&quot;"/>
     <numFmt numFmtId="166" formatCode="+0.0;-0.0"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -81,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -95,6 +96,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -460,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -555,85 +560,99 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <f>SUM(OFFSET(Quarterly!$F$1,MATCH($B$4,Quarterly!$A:$A,0),0,4,1))</f>
+        <f>XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$I:$I)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>(blank rate change = fewer than 4 quarters before the selection)</t>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Rate change vs same quarter a year earlier (pt)</t>
         </is>
       </c>
       <c r="B12" s="8">
-        <f>INDEX(Quarterly!$G:$G,MATCH($B$4,Quarterly!$A:$A,0))-INDEX(Quarterly!$G:$G,MATCH($B$4,Quarterly!$A:$A,0)+4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr"/>
+        <f>XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$J:$J)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>(blank 4-quarter sum = fewer than 4 quarters of history up to the selection; blank rate change = no same quarter a year earlier — formula-blank, never #REF)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Refresh: re-run the pipeline, then re-run this builder —</t>
-        </is>
-      </c>
+      <c r="A15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  python src/download.py --force     # or without --force if the raw files exist</t>
+          <t>Refresh: re-run the pipeline, then re-run this builder —</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  python src/build_dataset.py        # staging + checks → data/processed/quarterly.parquet</t>
+          <t xml:space="preserve">  python src/run_all.py             # everything in order (download → dataset → analysis → figures → workbook)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  python src/analysis.py             # bridge + sensitivity → outputs/*.csv</t>
+          <t xml:space="preserve">  python src/build_workbook.py      # just this file</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  python src/build_workbook.py       # this file</t>
-        </is>
-      </c>
+      <c r="A19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr"/>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>The 4-quarter and rate-change cells are keyed to the Seq column (1 = oldest) on the Quarterly sheet —</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Source: MAS credit &amp; charge cards via data.gov.sg — Singapore Open Data Licence. See docs/data_audit.md.</t>
+          <t>plain SUMIFS with a bounds guard: no OFFSET, and still correct if you re-sort the sheet.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Charge-off rate is as published: bad debts written off ÷ average rollover balance, annualised.</t>
+          <t>The Annual bridge sheet computes the split live with SUMIFS / AVERAGEIFS — it mirrors outputs/yearly_bridge.csv.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Formula-only, no macros. XLOOKUP needs Excel 2021+/365; in older readers swap it for the INDEX/MATCH pattern used below it.</t>
+          <t>Source: MAS credit &amp; charge cards via data.gov.sg — Singapore Open Data Licence. See docs/data_audit.md.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Charge-off rate is as published: bad debts written off ÷ average rollover balance, annualised.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Formula-only, no macros. XLOOKUP needs Excel 2021+/365; older readers can swap it for INDEX/MATCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>Numbers reproduce outputs/yearly_bridge.csv and the README headline for the same pull.</t>
         </is>
@@ -655,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -665,6 +684,9 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -703,6 +725,21 @@
           <t>Published rate (%)</t>
         </is>
       </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>Seq (1=oldest)</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>Last 4 qtrs: write-offs (S$M)</t>
+        </is>
+      </c>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>Rate chg vs yr earlier (pt)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -728,6 +765,17 @@
       <c r="G2" t="n">
         <v>5.9</v>
       </c>
+      <c r="H2" t="n">
+        <v>47</v>
+      </c>
+      <c r="I2">
+        <f>IF($H2&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H2-3,$H$2:$H$48,"&lt;="&amp;$H2),"")</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>IF($H2&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H2-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -753,6 +801,17 @@
       <c r="G3" t="n">
         <v>5.9</v>
       </c>
+      <c r="H3" t="n">
+        <v>46</v>
+      </c>
+      <c r="I3">
+        <f>IF($H3&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H3-3,$H$2:$H$48,"&lt;="&amp;$H3),"")</f>
+        <v/>
+      </c>
+      <c r="J3">
+        <f>IF($H3&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H3-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -778,6 +837,17 @@
       <c r="G4" t="n">
         <v>6</v>
       </c>
+      <c r="H4" t="n">
+        <v>45</v>
+      </c>
+      <c r="I4">
+        <f>IF($H4&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H4-3,$H$2:$H$48,"&lt;="&amp;$H4),"")</f>
+        <v/>
+      </c>
+      <c r="J4">
+        <f>IF($H4&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H4-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -803,6 +873,17 @@
       <c r="G5" t="n">
         <v>5.9</v>
       </c>
+      <c r="H5" t="n">
+        <v>44</v>
+      </c>
+      <c r="I5">
+        <f>IF($H5&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H5-3,$H$2:$H$48,"&lt;="&amp;$H5),"")</f>
+        <v/>
+      </c>
+      <c r="J5">
+        <f>IF($H5&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H5-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -828,6 +909,17 @@
       <c r="G6" t="n">
         <v>6</v>
       </c>
+      <c r="H6" t="n">
+        <v>43</v>
+      </c>
+      <c r="I6">
+        <f>IF($H6&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H6-3,$H$2:$H$48,"&lt;="&amp;$H6),"")</f>
+        <v/>
+      </c>
+      <c r="J6">
+        <f>IF($H6&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H6-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -853,6 +945,17 @@
       <c r="G7" t="n">
         <v>5.9</v>
       </c>
+      <c r="H7" t="n">
+        <v>42</v>
+      </c>
+      <c r="I7">
+        <f>IF($H7&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H7-3,$H$2:$H$48,"&lt;="&amp;$H7),"")</f>
+        <v/>
+      </c>
+      <c r="J7">
+        <f>IF($H7&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H7-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -878,6 +981,17 @@
       <c r="G8" t="n">
         <v>5.4</v>
       </c>
+      <c r="H8" t="n">
+        <v>41</v>
+      </c>
+      <c r="I8">
+        <f>IF($H8&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H8-3,$H$2:$H$48,"&lt;="&amp;$H8),"")</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>IF($H8&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H8-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -903,6 +1017,17 @@
       <c r="G9" t="n">
         <v>5.3</v>
       </c>
+      <c r="H9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I9">
+        <f>IF($H9&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H9-3,$H$2:$H$48,"&lt;="&amp;$H9),"")</f>
+        <v/>
+      </c>
+      <c r="J9">
+        <f>IF($H9&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H9-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -928,6 +1053,17 @@
       <c r="G10" t="n">
         <v>6.5</v>
       </c>
+      <c r="H10" t="n">
+        <v>39</v>
+      </c>
+      <c r="I10">
+        <f>IF($H10&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H10-3,$H$2:$H$48,"&lt;="&amp;$H10),"")</f>
+        <v/>
+      </c>
+      <c r="J10">
+        <f>IF($H10&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H10-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -953,6 +1089,17 @@
       <c r="G11" t="n">
         <v>5</v>
       </c>
+      <c r="H11" t="n">
+        <v>38</v>
+      </c>
+      <c r="I11">
+        <f>IF($H11&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H11-3,$H$2:$H$48,"&lt;="&amp;$H11),"")</f>
+        <v/>
+      </c>
+      <c r="J11">
+        <f>IF($H11&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H11-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -978,6 +1125,17 @@
       <c r="G12" t="n">
         <v>4.2</v>
       </c>
+      <c r="H12" t="n">
+        <v>37</v>
+      </c>
+      <c r="I12">
+        <f>IF($H12&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H12-3,$H$2:$H$48,"&lt;="&amp;$H12),"")</f>
+        <v/>
+      </c>
+      <c r="J12">
+        <f>IF($H12&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H12-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1003,6 +1161,17 @@
       <c r="G13" t="n">
         <v>4.5</v>
       </c>
+      <c r="H13" t="n">
+        <v>36</v>
+      </c>
+      <c r="I13">
+        <f>IF($H13&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H13-3,$H$2:$H$48,"&lt;="&amp;$H13),"")</f>
+        <v/>
+      </c>
+      <c r="J13">
+        <f>IF($H13&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H13-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1028,6 +1197,17 @@
       <c r="G14" t="n">
         <v>3.9</v>
       </c>
+      <c r="H14" t="n">
+        <v>35</v>
+      </c>
+      <c r="I14">
+        <f>IF($H14&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H14-3,$H$2:$H$48,"&lt;="&amp;$H14),"")</f>
+        <v/>
+      </c>
+      <c r="J14">
+        <f>IF($H14&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H14-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1053,6 +1233,17 @@
       <c r="G15" t="n">
         <v>3.7</v>
       </c>
+      <c r="H15" t="n">
+        <v>34</v>
+      </c>
+      <c r="I15">
+        <f>IF($H15&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H15-3,$H$2:$H$48,"&lt;="&amp;$H15),"")</f>
+        <v/>
+      </c>
+      <c r="J15">
+        <f>IF($H15&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H15-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1078,6 +1269,17 @@
       <c r="G16" t="n">
         <v>3.4</v>
       </c>
+      <c r="H16" t="n">
+        <v>33</v>
+      </c>
+      <c r="I16">
+        <f>IF($H16&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H16-3,$H$2:$H$48,"&lt;="&amp;$H16),"")</f>
+        <v/>
+      </c>
+      <c r="J16">
+        <f>IF($H16&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H16-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1103,6 +1305,17 @@
       <c r="G17" t="n">
         <v>3.5</v>
       </c>
+      <c r="H17" t="n">
+        <v>32</v>
+      </c>
+      <c r="I17">
+        <f>IF($H17&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H17-3,$H$2:$H$48,"&lt;="&amp;$H17),"")</f>
+        <v/>
+      </c>
+      <c r="J17">
+        <f>IF($H17&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H17-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1128,6 +1341,17 @@
       <c r="G18" t="n">
         <v>3.5</v>
       </c>
+      <c r="H18" t="n">
+        <v>31</v>
+      </c>
+      <c r="I18">
+        <f>IF($H18&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H18-3,$H$2:$H$48,"&lt;="&amp;$H18),"")</f>
+        <v/>
+      </c>
+      <c r="J18">
+        <f>IF($H18&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H18-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1153,6 +1377,17 @@
       <c r="G19" t="n">
         <v>4.1</v>
       </c>
+      <c r="H19" t="n">
+        <v>30</v>
+      </c>
+      <c r="I19">
+        <f>IF($H19&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H19-3,$H$2:$H$48,"&lt;="&amp;$H19),"")</f>
+        <v/>
+      </c>
+      <c r="J19">
+        <f>IF($H19&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H19-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1178,6 +1413,17 @@
       <c r="G20" t="n">
         <v>4.4</v>
       </c>
+      <c r="H20" t="n">
+        <v>29</v>
+      </c>
+      <c r="I20">
+        <f>IF($H20&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H20-3,$H$2:$H$48,"&lt;="&amp;$H20),"")</f>
+        <v/>
+      </c>
+      <c r="J20">
+        <f>IF($H20&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H20-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1203,6 +1449,17 @@
       <c r="G21" t="n">
         <v>4.8</v>
       </c>
+      <c r="H21" t="n">
+        <v>28</v>
+      </c>
+      <c r="I21">
+        <f>IF($H21&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H21-3,$H$2:$H$48,"&lt;="&amp;$H21),"")</f>
+        <v/>
+      </c>
+      <c r="J21">
+        <f>IF($H21&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H21-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1228,6 +1485,17 @@
       <c r="G22" t="n">
         <v>4.1</v>
       </c>
+      <c r="H22" t="n">
+        <v>27</v>
+      </c>
+      <c r="I22">
+        <f>IF($H22&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H22-3,$H$2:$H$48,"&lt;="&amp;$H22),"")</f>
+        <v/>
+      </c>
+      <c r="J22">
+        <f>IF($H22&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H22-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1253,6 +1521,17 @@
       <c r="G23" t="n">
         <v>5</v>
       </c>
+      <c r="H23" t="n">
+        <v>26</v>
+      </c>
+      <c r="I23">
+        <f>IF($H23&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H23-3,$H$2:$H$48,"&lt;="&amp;$H23),"")</f>
+        <v/>
+      </c>
+      <c r="J23">
+        <f>IF($H23&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H23-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1278,6 +1557,17 @@
       <c r="G24" t="n">
         <v>6.1</v>
       </c>
+      <c r="H24" t="n">
+        <v>25</v>
+      </c>
+      <c r="I24">
+        <f>IF($H24&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H24-3,$H$2:$H$48,"&lt;="&amp;$H24),"")</f>
+        <v/>
+      </c>
+      <c r="J24">
+        <f>IF($H24&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H24-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1303,6 +1593,17 @@
       <c r="G25" t="n">
         <v>9.1</v>
       </c>
+      <c r="H25" t="n">
+        <v>24</v>
+      </c>
+      <c r="I25">
+        <f>IF($H25&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H25-3,$H$2:$H$48,"&lt;="&amp;$H25),"")</f>
+        <v/>
+      </c>
+      <c r="J25">
+        <f>IF($H25&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H25-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1328,6 +1629,17 @@
       <c r="G26" t="n">
         <v>7.3</v>
       </c>
+      <c r="H26" t="n">
+        <v>23</v>
+      </c>
+      <c r="I26">
+        <f>IF($H26&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H26-3,$H$2:$H$48,"&lt;="&amp;$H26),"")</f>
+        <v/>
+      </c>
+      <c r="J26">
+        <f>IF($H26&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H26-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1353,6 +1665,17 @@
       <c r="G27" t="n">
         <v>6.7</v>
       </c>
+      <c r="H27" t="n">
+        <v>22</v>
+      </c>
+      <c r="I27">
+        <f>IF($H27&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H27-3,$H$2:$H$48,"&lt;="&amp;$H27),"")</f>
+        <v/>
+      </c>
+      <c r="J27">
+        <f>IF($H27&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H27-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1378,6 +1701,17 @@
       <c r="G28" t="n">
         <v>6.3</v>
       </c>
+      <c r="H28" t="n">
+        <v>21</v>
+      </c>
+      <c r="I28">
+        <f>IF($H28&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H28-3,$H$2:$H$48,"&lt;="&amp;$H28),"")</f>
+        <v/>
+      </c>
+      <c r="J28">
+        <f>IF($H28&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H28-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1403,6 +1737,17 @@
       <c r="G29" t="n">
         <v>5.9</v>
       </c>
+      <c r="H29" t="n">
+        <v>20</v>
+      </c>
+      <c r="I29">
+        <f>IF($H29&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H29-3,$H$2:$H$48,"&lt;="&amp;$H29),"")</f>
+        <v/>
+      </c>
+      <c r="J29">
+        <f>IF($H29&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H29-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1428,6 +1773,17 @@
       <c r="G30" t="n">
         <v>5.7</v>
       </c>
+      <c r="H30" t="n">
+        <v>19</v>
+      </c>
+      <c r="I30">
+        <f>IF($H30&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H30-3,$H$2:$H$48,"&lt;="&amp;$H30),"")</f>
+        <v/>
+      </c>
+      <c r="J30">
+        <f>IF($H30&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H30-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1453,6 +1809,17 @@
       <c r="G31" t="n">
         <v>6.1</v>
       </c>
+      <c r="H31" t="n">
+        <v>18</v>
+      </c>
+      <c r="I31">
+        <f>IF($H31&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H31-3,$H$2:$H$48,"&lt;="&amp;$H31),"")</f>
+        <v/>
+      </c>
+      <c r="J31">
+        <f>IF($H31&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H31-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1478,6 +1845,17 @@
       <c r="G32" t="n">
         <v>6</v>
       </c>
+      <c r="H32" t="n">
+        <v>17</v>
+      </c>
+      <c r="I32">
+        <f>IF($H32&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H32-3,$H$2:$H$48,"&lt;="&amp;$H32),"")</f>
+        <v/>
+      </c>
+      <c r="J32">
+        <f>IF($H32&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H32-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1503,6 +1881,17 @@
       <c r="G33" t="n">
         <v>6.1</v>
       </c>
+      <c r="H33" t="n">
+        <v>16</v>
+      </c>
+      <c r="I33">
+        <f>IF($H33&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H33-3,$H$2:$H$48,"&lt;="&amp;$H33),"")</f>
+        <v/>
+      </c>
+      <c r="J33">
+        <f>IF($H33&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H33-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1528,6 +1917,17 @@
       <c r="G34" t="n">
         <v>6.3</v>
       </c>
+      <c r="H34" t="n">
+        <v>15</v>
+      </c>
+      <c r="I34">
+        <f>IF($H34&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H34-3,$H$2:$H$48,"&lt;="&amp;$H34),"")</f>
+        <v/>
+      </c>
+      <c r="J34">
+        <f>IF($H34&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H34-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1553,6 +1953,17 @@
       <c r="G35" t="n">
         <v>6.2</v>
       </c>
+      <c r="H35" t="n">
+        <v>14</v>
+      </c>
+      <c r="I35">
+        <f>IF($H35&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H35-3,$H$2:$H$48,"&lt;="&amp;$H35),"")</f>
+        <v/>
+      </c>
+      <c r="J35">
+        <f>IF($H35&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H35-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1578,6 +1989,17 @@
       <c r="G36" t="n">
         <v>4.8</v>
       </c>
+      <c r="H36" t="n">
+        <v>13</v>
+      </c>
+      <c r="I36">
+        <f>IF($H36&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H36-3,$H$2:$H$48,"&lt;="&amp;$H36),"")</f>
+        <v/>
+      </c>
+      <c r="J36">
+        <f>IF($H36&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H36-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1603,6 +2025,17 @@
       <c r="G37" t="n">
         <v>4.4</v>
       </c>
+      <c r="H37" t="n">
+        <v>12</v>
+      </c>
+      <c r="I37">
+        <f>IF($H37&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H37-3,$H$2:$H$48,"&lt;="&amp;$H37),"")</f>
+        <v/>
+      </c>
+      <c r="J37">
+        <f>IF($H37&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H37-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1628,6 +2061,17 @@
       <c r="G38" t="n">
         <v>4.8</v>
       </c>
+      <c r="H38" t="n">
+        <v>11</v>
+      </c>
+      <c r="I38">
+        <f>IF($H38&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H38-3,$H$2:$H$48,"&lt;="&amp;$H38),"")</f>
+        <v/>
+      </c>
+      <c r="J38">
+        <f>IF($H38&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H38-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1653,6 +2097,17 @@
       <c r="G39" t="n">
         <v>5.3</v>
       </c>
+      <c r="H39" t="n">
+        <v>10</v>
+      </c>
+      <c r="I39">
+        <f>IF($H39&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H39-3,$H$2:$H$48,"&lt;="&amp;$H39),"")</f>
+        <v/>
+      </c>
+      <c r="J39">
+        <f>IF($H39&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H39-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1678,6 +2133,17 @@
       <c r="G40" t="n">
         <v>5</v>
       </c>
+      <c r="H40" t="n">
+        <v>9</v>
+      </c>
+      <c r="I40">
+        <f>IF($H40&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H40-3,$H$2:$H$48,"&lt;="&amp;$H40),"")</f>
+        <v/>
+      </c>
+      <c r="J40">
+        <f>IF($H40&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H40-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1703,6 +2169,17 @@
       <c r="G41" t="n">
         <v>5</v>
       </c>
+      <c r="H41" t="n">
+        <v>8</v>
+      </c>
+      <c r="I41">
+        <f>IF($H41&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H41-3,$H$2:$H$48,"&lt;="&amp;$H41),"")</f>
+        <v/>
+      </c>
+      <c r="J41">
+        <f>IF($H41&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H41-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1728,6 +2205,17 @@
       <c r="G42" t="n">
         <v>4.7</v>
       </c>
+      <c r="H42" t="n">
+        <v>7</v>
+      </c>
+      <c r="I42">
+        <f>IF($H42&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H42-3,$H$2:$H$48,"&lt;="&amp;$H42),"")</f>
+        <v/>
+      </c>
+      <c r="J42">
+        <f>IF($H42&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H42-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1753,6 +2241,17 @@
       <c r="G43" t="n">
         <v>5.2</v>
       </c>
+      <c r="H43" t="n">
+        <v>6</v>
+      </c>
+      <c r="I43">
+        <f>IF($H43&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H43-3,$H$2:$H$48,"&lt;="&amp;$H43),"")</f>
+        <v/>
+      </c>
+      <c r="J43">
+        <f>IF($H43&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H43-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1778,6 +2277,17 @@
       <c r="G44" t="n">
         <v>6.2</v>
       </c>
+      <c r="H44" t="n">
+        <v>5</v>
+      </c>
+      <c r="I44">
+        <f>IF($H44&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H44-3,$H$2:$H$48,"&lt;="&amp;$H44),"")</f>
+        <v/>
+      </c>
+      <c r="J44">
+        <f>IF($H44&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H44-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1803,6 +2313,17 @@
       <c r="G45" t="n">
         <v>6.1</v>
       </c>
+      <c r="H45" t="n">
+        <v>4</v>
+      </c>
+      <c r="I45">
+        <f>IF($H45&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H45-3,$H$2:$H$48,"&lt;="&amp;$H45),"")</f>
+        <v/>
+      </c>
+      <c r="J45">
+        <f>IF($H45&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H45-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1828,6 +2349,17 @@
       <c r="G46" t="n">
         <v>5.4</v>
       </c>
+      <c r="H46" t="n">
+        <v>3</v>
+      </c>
+      <c r="I46">
+        <f>IF($H46&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H46-3,$H$2:$H$48,"&lt;="&amp;$H46),"")</f>
+        <v/>
+      </c>
+      <c r="J46">
+        <f>IF($H46&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H46-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1853,6 +2385,17 @@
       <c r="G47" t="n">
         <v>5.5</v>
       </c>
+      <c r="H47" t="n">
+        <v>2</v>
+      </c>
+      <c r="I47">
+        <f>IF($H47&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H47-3,$H$2:$H$48,"&lt;="&amp;$H47),"")</f>
+        <v/>
+      </c>
+      <c r="J47">
+        <f>IF($H47&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H47-4),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1877,6 +2420,17 @@
       </c>
       <c r="G48" t="n">
         <v>5.2</v>
+      </c>
+      <c r="H48" t="n">
+        <v>1</v>
+      </c>
+      <c r="I48">
+        <f>IF($H48&gt;=4,SUMIFS($F$2:$F$48,$H$2:$H$48,"&gt;="&amp;$H48-3,$H$2:$H$48,"&lt;="&amp;$H48),"")</f>
+        <v/>
+      </c>
+      <c r="J48">
+        <f>IF($H48&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H48-4),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1890,20 +2444,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1914,52 +2466,42 @@
       </c>
       <c r="B1" s="10" t="inlineStr">
         <is>
-          <t>vs year</t>
+          <t>Write-offs (S$M)</t>
         </is>
       </c>
       <c r="C1" s="10" t="inlineStr">
         <is>
-          <t>Write-offs (S$M)</t>
+          <t>Avg rollover (S$M)</t>
         </is>
       </c>
       <c r="D1" s="10" t="inlineStr">
         <is>
-          <t>Avg rollover (S$M)</t>
+          <t>Rate, recomputed (%)</t>
         </is>
       </c>
       <c r="E1" s="10" t="inlineStr">
         <is>
-          <t>Rate, recomputed (%)</t>
+          <t>Rate, published (%)</t>
         </is>
       </c>
       <c r="F1" s="10" t="inlineStr">
         <is>
-          <t>Rate, published (%)</t>
+          <t>Δ write-offs (S$M)</t>
         </is>
       </c>
       <c r="G1" s="10" t="inlineStr">
         <is>
-          <t>Δ write-offs (S$M)</t>
+          <t>Volume effect (S$M)</t>
         </is>
       </c>
       <c r="H1" s="10" t="inlineStr">
         <is>
-          <t>Volume effect (S$M)</t>
+          <t>Rate effect (S$M)</t>
         </is>
       </c>
       <c r="I1" s="10" t="inlineStr">
         <is>
-          <t>Rate effect (S$M)</t>
-        </is>
-      </c>
-      <c r="J1" s="10" t="inlineStr">
-        <is>
-          <t>Interaction (S$M)</t>
-        </is>
-      </c>
-      <c r="K1" s="10" t="inlineStr">
-        <is>
-          <t>Check sum (S$M)</t>
+          <t>Closure (Δ−vol−rate, 0 = exact)</t>
         </is>
       </c>
     </row>
@@ -1967,350 +2509,362 @@
       <c r="A2" t="n">
         <v>2016</v>
       </c>
-      <c r="B2" t="n">
-        <v>2015</v>
-      </c>
-      <c r="C2" t="n">
-        <v>296.5</v>
-      </c>
-      <c r="D2" t="n">
-        <v>6089.62</v>
-      </c>
-      <c r="E2" t="n">
-        <v>4.869</v>
-      </c>
-      <c r="F2" t="n">
+      <c r="B2" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A2)</f>
+        <v/>
+      </c>
+      <c r="C2" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A2)</f>
+        <v/>
+      </c>
+      <c r="D2" s="12">
+        <f>B2/C2*100</f>
+        <v/>
+      </c>
+      <c r="E2" s="11" t="n">
         <v>4.9</v>
       </c>
-      <c r="G2" t="n">
-        <v>-44.3</v>
-      </c>
-      <c r="H2" t="n">
-        <v>5.24</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-49.54</v>
-      </c>
-      <c r="J2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>-44.3</v>
-      </c>
+      <c r="F2" s="13" t="n"/>
+      <c r="G2" s="13" t="n"/>
+      <c r="H2" s="13" t="n"/>
+      <c r="I2" s="14" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2017</v>
       </c>
-      <c r="B3" t="n">
-        <v>2016</v>
-      </c>
-      <c r="C3" t="n">
-        <v>288.3</v>
-      </c>
-      <c r="D3" t="n">
-        <v>6085.6</v>
-      </c>
-      <c r="E3" t="n">
-        <v>4.737</v>
-      </c>
-      <c r="F3" t="n">
+      <c r="B3" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A3)</f>
+        <v/>
+      </c>
+      <c r="C3" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A3)</f>
+        <v/>
+      </c>
+      <c r="D3" s="12">
+        <f>B3/C3*100</f>
+        <v/>
+      </c>
+      <c r="E3" s="11" t="n">
         <v>4.7</v>
       </c>
-      <c r="G3" t="n">
-        <v>-8.199999999999999</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-0.19</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-8.01</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>-8.199999999999999</v>
+      <c r="F3" s="13">
+        <f>B3-B2</f>
+        <v/>
+      </c>
+      <c r="G3" s="13">
+        <f>(C3-C2)*(D2+D3)/200</f>
+        <v/>
+      </c>
+      <c r="H3" s="13">
+        <f>(D3-D2)/100*(C2+C3)/2</f>
+        <v/>
+      </c>
+      <c r="I3" s="14">
+        <f>IF(F3="","",ROUND(F3-G3-H3,6))</f>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>2018</v>
       </c>
-      <c r="B4" t="n">
-        <v>2017</v>
-      </c>
-      <c r="C4" t="n">
-        <v>366.5</v>
-      </c>
-      <c r="D4" t="n">
-        <v>6121.3</v>
-      </c>
-      <c r="E4" t="n">
-        <v>5.987</v>
-      </c>
-      <c r="F4" t="n">
+      <c r="B4" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A4)</f>
+        <v/>
+      </c>
+      <c r="C4" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A4)</f>
+        <v/>
+      </c>
+      <c r="D4" s="12">
+        <f>B4/C4*100</f>
+        <v/>
+      </c>
+      <c r="E4" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="G4" t="n">
-        <v>78.2</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="I4" t="n">
-        <v>76.29000000000001</v>
-      </c>
-      <c r="J4" t="n">
-        <v>-0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>78.2</v>
+      <c r="F4" s="13">
+        <f>B4-B3</f>
+        <v/>
+      </c>
+      <c r="G4" s="13">
+        <f>(C4-C3)*(D3+D4)/200</f>
+        <v/>
+      </c>
+      <c r="H4" s="13">
+        <f>(D4-D3)/100*(C3+C4)/2</f>
+        <v/>
+      </c>
+      <c r="I4" s="14">
+        <f>IF(F4="","",ROUND(F4-G4-H4,6))</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>2019</v>
       </c>
-      <c r="B5" t="n">
-        <v>2018</v>
-      </c>
-      <c r="C5" t="n">
-        <v>364.9</v>
-      </c>
-      <c r="D5" t="n">
-        <v>6239.18</v>
-      </c>
-      <c r="E5" t="n">
-        <v>5.849</v>
-      </c>
-      <c r="F5" t="n">
+      <c r="B5" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A5)</f>
+        <v/>
+      </c>
+      <c r="C5" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A5)</f>
+        <v/>
+      </c>
+      <c r="D5" s="12">
+        <f>B5/C5*100</f>
+        <v/>
+      </c>
+      <c r="E5" s="11" t="n">
         <v>5.8</v>
       </c>
-      <c r="G5" t="n">
-        <v>-1.6</v>
-      </c>
-      <c r="H5" t="n">
-        <v>6.98</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-8.58</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>-1.6</v>
+      <c r="F5" s="13">
+        <f>B5-B4</f>
+        <v/>
+      </c>
+      <c r="G5" s="13">
+        <f>(C5-C4)*(D4+D5)/200</f>
+        <v/>
+      </c>
+      <c r="H5" s="13">
+        <f>(D5-D4)/100*(C4+C5)/2</f>
+        <v/>
+      </c>
+      <c r="I5" s="14">
+        <f>IF(F5="","",ROUND(F5-G5-H5,6))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>2020</v>
       </c>
-      <c r="B6" t="n">
-        <v>2019</v>
-      </c>
-      <c r="C6" t="n">
-        <v>396.7</v>
-      </c>
-      <c r="D6" t="n">
-        <v>5601.88</v>
-      </c>
-      <c r="E6" t="n">
-        <v>7.082</v>
-      </c>
-      <c r="F6" t="n">
+      <c r="B6" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A6)</f>
+        <v/>
+      </c>
+      <c r="C6" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A6)</f>
+        <v/>
+      </c>
+      <c r="D6" s="12">
+        <f>B6/C6*100</f>
+        <v/>
+      </c>
+      <c r="E6" s="11" t="n">
         <v>7.1</v>
       </c>
-      <c r="G6" t="n">
-        <v>31.8</v>
-      </c>
-      <c r="H6" t="n">
-        <v>-41.2</v>
-      </c>
-      <c r="I6" t="n">
-        <v>73</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>31.8</v>
+      <c r="F6" s="13">
+        <f>B6-B5</f>
+        <v/>
+      </c>
+      <c r="G6" s="13">
+        <f>(C6-C5)*(D5+D6)/200</f>
+        <v/>
+      </c>
+      <c r="H6" s="13">
+        <f>(D6-D5)/100*(C5+C6)/2</f>
+        <v/>
+      </c>
+      <c r="I6" s="14">
+        <f>IF(F6="","",ROUND(F6-G6-H6,6))</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
         <v>2021</v>
       </c>
-      <c r="B7" t="n">
-        <v>2020</v>
-      </c>
-      <c r="C7" t="n">
-        <v>234.6</v>
-      </c>
-      <c r="D7" t="n">
-        <v>5231.02</v>
-      </c>
-      <c r="E7" t="n">
-        <v>4.485</v>
-      </c>
-      <c r="F7" t="n">
+      <c r="B7" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A7)</f>
+        <v/>
+      </c>
+      <c r="C7" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A7)</f>
+        <v/>
+      </c>
+      <c r="D7" s="12">
+        <f>B7/C7*100</f>
+        <v/>
+      </c>
+      <c r="E7" s="11" t="n">
         <v>4.5</v>
       </c>
-      <c r="G7" t="n">
-        <v>-162.1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>-21.45</v>
-      </c>
-      <c r="I7" t="n">
-        <v>-140.65</v>
-      </c>
-      <c r="J7" t="n">
-        <v>-0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>-162.1</v>
+      <c r="F7" s="13">
+        <f>B7-B6</f>
+        <v/>
+      </c>
+      <c r="G7" s="13">
+        <f>(C7-C6)*(D6+D7)/200</f>
+        <v/>
+      </c>
+      <c r="H7" s="13">
+        <f>(D7-D6)/100*(C6+C7)/2</f>
+        <v/>
+      </c>
+      <c r="I7" s="14">
+        <f>IF(F7="","",ROUND(F7-G7-H7,6))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
         <v>2022</v>
       </c>
-      <c r="B8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C8" t="n">
-        <v>201.9</v>
-      </c>
-      <c r="D8" t="n">
-        <v>5708.5</v>
-      </c>
-      <c r="E8" t="n">
-        <v>3.537</v>
-      </c>
-      <c r="F8" t="n">
+      <c r="B8" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="12">
+        <f>B8/C8*100</f>
+        <v/>
+      </c>
+      <c r="E8" s="11" t="n">
         <v>3.5</v>
       </c>
-      <c r="G8" t="n">
-        <v>-32.7</v>
-      </c>
-      <c r="H8" t="n">
-        <v>19.15</v>
-      </c>
-      <c r="I8" t="n">
-        <v>-51.85</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>-32.7</v>
+      <c r="F8" s="13">
+        <f>B8-B7</f>
+        <v/>
+      </c>
+      <c r="G8" s="13">
+        <f>(C8-C7)*(D7+D8)/200</f>
+        <v/>
+      </c>
+      <c r="H8" s="13">
+        <f>(D8-D7)/100*(C7+C8)/2</f>
+        <v/>
+      </c>
+      <c r="I8" s="14">
+        <f>IF(F8="","",ROUND(F8-G8-H8,6))</f>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>2023</v>
       </c>
-      <c r="B9" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C9" t="n">
-        <v>270.4</v>
-      </c>
-      <c r="D9" t="n">
-        <v>6728.45</v>
-      </c>
-      <c r="E9" t="n">
-        <v>4.019</v>
-      </c>
-      <c r="F9" t="n">
+      <c r="B9" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A9)</f>
+        <v/>
+      </c>
+      <c r="D9" s="12">
+        <f>B9/C9*100</f>
+        <v/>
+      </c>
+      <c r="E9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G9" t="n">
-        <v>68.5</v>
-      </c>
-      <c r="H9" t="n">
-        <v>38.53</v>
-      </c>
-      <c r="I9" t="n">
-        <v>29.97</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>68.5</v>
+      <c r="F9" s="13">
+        <f>B9-B8</f>
+        <v/>
+      </c>
+      <c r="G9" s="13">
+        <f>(C9-C8)*(D8+D9)/200</f>
+        <v/>
+      </c>
+      <c r="H9" s="13">
+        <f>(D9-D8)/100*(C8+C9)/2</f>
+        <v/>
+      </c>
+      <c r="I9" s="14">
+        <f>IF(F9="","",ROUND(F9-G9-H9,6))</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
         <v>2024</v>
       </c>
-      <c r="B10" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C10" t="n">
-        <v>423.2</v>
-      </c>
-      <c r="D10" t="n">
-        <v>7785.47</v>
-      </c>
-      <c r="E10" t="n">
-        <v>5.436</v>
-      </c>
-      <c r="F10" t="n">
+      <c r="B10" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A10)</f>
+        <v/>
+      </c>
+      <c r="D10" s="12">
+        <f>B10/C10*100</f>
+        <v/>
+      </c>
+      <c r="E10" s="11" t="n">
         <v>5.4</v>
       </c>
-      <c r="G10" t="n">
-        <v>152.8</v>
-      </c>
-      <c r="H10" t="n">
-        <v>49.97</v>
-      </c>
-      <c r="I10" t="n">
-        <v>102.83</v>
-      </c>
-      <c r="J10" t="n">
-        <v>-0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>152.8</v>
+      <c r="F10" s="13">
+        <f>B10-B9</f>
+        <v/>
+      </c>
+      <c r="G10" s="13">
+        <f>(C10-C9)*(D9+D10)/200</f>
+        <v/>
+      </c>
+      <c r="H10" s="13">
+        <f>(D10-D9)/100*(C9+C10)/2</f>
+        <v/>
+      </c>
+      <c r="I10" s="14">
+        <f>IF(F10="","",ROUND(F10-G10-H10,6))</f>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
         <v>2025</v>
       </c>
-      <c r="B11" t="n">
-        <v>2024</v>
-      </c>
-      <c r="C11" t="n">
-        <v>519.7</v>
-      </c>
-      <c r="D11" t="n">
-        <v>8920.299999999999</v>
-      </c>
-      <c r="E11" t="n">
-        <v>5.826</v>
-      </c>
-      <c r="F11" t="n">
+      <c r="B11" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A11)</f>
+        <v/>
+      </c>
+      <c r="D11" s="12">
+        <f>B11/C11*100</f>
+        <v/>
+      </c>
+      <c r="E11" s="11" t="n">
         <v>5.8</v>
       </c>
-      <c r="G11" t="n">
-        <v>96.5</v>
-      </c>
-      <c r="H11" t="n">
-        <v>63.9</v>
-      </c>
-      <c r="I11" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>96.5</v>
+      <c r="F11" s="13">
+        <f>B11-B10</f>
+        <v/>
+      </c>
+      <c r="G11" s="13">
+        <f>(C11-C10)*(D10+D11)/200</f>
+        <v/>
+      </c>
+      <c r="H11" s="13">
+        <f>(D11-D10)/100*(C10+C11)/2</f>
+        <v/>
+      </c>
+      <c r="I11" s="14">
+        <f>IF(F11="","",ROUND(F11-G11-H11,6))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Live formulas from the Quarterly sheet (SUMIFS / AVERAGEIFS) — the same midpoint split as outputs/yearly_bridge.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Column E (published rate) is pasted from the MAS annual file; volume = Δrollover × avg rate · rate = Δrate × avg rollover.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: resolve external review findings and harden artifact validation
</commit_message>
<xml_diff>
--- a/outputs/quick_check.xlsx
+++ b/outputs/quick_check.xlsx
@@ -11,7 +11,15 @@
     <sheet name="Quarterly" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Annual bridge" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quick check'!$A$1:$B$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Quarterly'!$A$1:$J$48</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Quarterly'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Quarterly'!$A$1:$J$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Annual bridge'!$A$1:$I$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Annual bridge'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Annual bridge'!$A$1:$I$15</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -84,18 +92,26 @@
   </cellStyleXfs>
   <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,6 +190,43 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="QuarterlyData" displayName="QuarterlyData" ref="A1:J48" headerRowCount="1">
+  <autoFilter ref="A1:J48"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Quarter"/>
+    <tableColumn id="2" name="Year"/>
+    <tableColumn id="3" name="Qtr"/>
+    <tableColumn id="4" name="Total billings (S$M)"/>
+    <tableColumn id="5" name="Rollover balance (S$M)"/>
+    <tableColumn id="6" name="Write-offs (S$M)"/>
+    <tableColumn id="7" name="Published rate (%)"/>
+    <tableColumn id="8" name="Seq (1=oldest)"/>
+    <tableColumn id="9" name="Last 4 qtrs: write-offs (S$M)"/>
+    <tableColumn id="10" name="Rate chg vs yr earlier (pt)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AnnualBridgeData" displayName="AnnualBridgeData" ref="A1:I12" headerRowCount="1">
+  <autoFilter ref="A1:I12"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Year"/>
+    <tableColumn id="2" name="Write-offs (S$M)"/>
+    <tableColumn id="3" name="Avg rollover (S$M)"/>
+    <tableColumn id="4" name="Rate, recomputed (%)"/>
+    <tableColumn id="5" name="Rate, published (%)"/>
+    <tableColumn id="6" name="Δ write-offs (S$M)"/>
+    <tableColumn id="7" name="Volume effect (S$M)"/>
+    <tableColumn id="8" name="Rate effect (S$M)"/>
+    <tableColumn id="9" name="Closure (Δ−vol−rate, 0 = exact)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -463,7 +516,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -472,14 +525,14 @@
     <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Card book — quick check (MAS credit &amp; charge cards, quarterly)</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>All issuers in Singapore, not one bank. Values S$M unless stated. Pick a quarter below — the block updates (formulas, no macros).</t>
@@ -498,8 +551,8 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
@@ -509,162 +562,180 @@
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Total billings (S$M, that quarter)</t>
         </is>
       </c>
-      <c r="B7" s="6">
-        <f>XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$D:$D)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="B7" s="7">
+        <f>_xlfn.XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$D:$D,"Invalid quarter")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Rollover balance (S$M, quarter-end)</t>
         </is>
       </c>
-      <c r="B8" s="6">
-        <f>XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$E:$E)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="B8" s="7">
+        <f>_xlfn.XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$E:$E,"Invalid quarter")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Write-offs (S$M, that quarter)</t>
         </is>
       </c>
-      <c r="B9" s="6">
-        <f>XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$F:$F)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="B9" s="7">
+        <f>_xlfn.XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$F:$F,"Invalid quarter")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Published charge-off rate (%, annualised)</t>
         </is>
       </c>
-      <c r="B10" s="7">
-        <f>XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$G:$G)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="B10" s="8">
+        <f>_xlfn.XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$G:$G,"Invalid quarter")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Write-offs, last 4 quarters incl. selected (S$M)</t>
         </is>
       </c>
-      <c r="B11" s="6">
-        <f>XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$I:$I)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="B11" s="7">
+        <f>_xlfn.XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$I:$I,"Invalid quarter")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Rate change vs same quarter a year earlier (pt)</t>
         </is>
       </c>
-      <c r="B12" s="8">
-        <f>XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$J:$J)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
+      <c r="B12" s="9">
+        <f>_xlfn.XLOOKUP($B$4,Quarterly!$A:$A,Quarterly!$J:$J,"Invalid quarter")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>(blank 4-quarter sum = fewer than 4 quarters of history up to the selection; blank rate change = no same quarter a year earlier — formula-blank, never #REF)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Refresh: re-run the pipeline, then re-run this builder —</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  python src/run_all.py             # everything in order (download → dataset → analysis → figures → workbook)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  python src/build_workbook.py      # just this file</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>The 4-quarter and rate-change cells are keyed to the Seq column (1 = oldest) on the Quarterly sheet —</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>plain SUMIFS with a bounds guard: no OFFSET, and still correct if you re-sort the sheet.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>The Annual bridge sheet computes the split live with SUMIFS / AVERAGEIFS — it mirrors outputs/yearly_bridge.csv.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Source: MAS credit &amp; charge cards via data.gov.sg — Singapore Open Data Licence. See docs/data_audit.md.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Charge-off rate is as published: bad debts written off ÷ average rollover balance, annualised.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Formula-only, no macros. XLOOKUP needs Excel 2021+/365; older readers can swap it for INDEX/MATCH.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Numbers reproduce outputs/yearly_bridge.csv and the README headline for the same pull.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A22:B22"/>
+  </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Pick a quarter from the list" type="list">
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Pick a quarter from the list" type="list" errorStyle="stop">
       <formula1>Quarterly!$A$2:$A$48</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -672,7 +743,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -689,7 +760,7 @@
     <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Quarter</t>
@@ -773,7 +844,7 @@
         <v/>
       </c>
       <c r="J2">
-        <f>IF($H2&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H2-4),"")</f>
+        <f>IF($H2&gt;=5,$G2-SUMIFS($G$2:$G$48,$H$2:$H$48,$H2-4),"")</f>
         <v/>
       </c>
     </row>
@@ -809,7 +880,7 @@
         <v/>
       </c>
       <c r="J3">
-        <f>IF($H3&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H3-4),"")</f>
+        <f>IF($H3&gt;=5,$G3-SUMIFS($G$2:$G$48,$H$2:$H$48,$H3-4),"")</f>
         <v/>
       </c>
     </row>
@@ -845,7 +916,7 @@
         <v/>
       </c>
       <c r="J4">
-        <f>IF($H4&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H4-4),"")</f>
+        <f>IF($H4&gt;=5,$G4-SUMIFS($G$2:$G$48,$H$2:$H$48,$H4-4),"")</f>
         <v/>
       </c>
     </row>
@@ -881,7 +952,7 @@
         <v/>
       </c>
       <c r="J5">
-        <f>IF($H5&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H5-4),"")</f>
+        <f>IF($H5&gt;=5,$G5-SUMIFS($G$2:$G$48,$H$2:$H$48,$H5-4),"")</f>
         <v/>
       </c>
     </row>
@@ -917,7 +988,7 @@
         <v/>
       </c>
       <c r="J6">
-        <f>IF($H6&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H6-4),"")</f>
+        <f>IF($H6&gt;=5,$G6-SUMIFS($G$2:$G$48,$H$2:$H$48,$H6-4),"")</f>
         <v/>
       </c>
     </row>
@@ -953,7 +1024,7 @@
         <v/>
       </c>
       <c r="J7">
-        <f>IF($H7&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H7-4),"")</f>
+        <f>IF($H7&gt;=5,$G7-SUMIFS($G$2:$G$48,$H$2:$H$48,$H7-4),"")</f>
         <v/>
       </c>
     </row>
@@ -989,7 +1060,7 @@
         <v/>
       </c>
       <c r="J8">
-        <f>IF($H8&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H8-4),"")</f>
+        <f>IF($H8&gt;=5,$G8-SUMIFS($G$2:$G$48,$H$2:$H$48,$H8-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1025,7 +1096,7 @@
         <v/>
       </c>
       <c r="J9">
-        <f>IF($H9&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H9-4),"")</f>
+        <f>IF($H9&gt;=5,$G9-SUMIFS($G$2:$G$48,$H$2:$H$48,$H9-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1061,7 +1132,7 @@
         <v/>
       </c>
       <c r="J10">
-        <f>IF($H10&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H10-4),"")</f>
+        <f>IF($H10&gt;=5,$G10-SUMIFS($G$2:$G$48,$H$2:$H$48,$H10-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1097,7 +1168,7 @@
         <v/>
       </c>
       <c r="J11">
-        <f>IF($H11&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H11-4),"")</f>
+        <f>IF($H11&gt;=5,$G11-SUMIFS($G$2:$G$48,$H$2:$H$48,$H11-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1133,7 +1204,7 @@
         <v/>
       </c>
       <c r="J12">
-        <f>IF($H12&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H12-4),"")</f>
+        <f>IF($H12&gt;=5,$G12-SUMIFS($G$2:$G$48,$H$2:$H$48,$H12-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1169,7 +1240,7 @@
         <v/>
       </c>
       <c r="J13">
-        <f>IF($H13&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H13-4),"")</f>
+        <f>IF($H13&gt;=5,$G13-SUMIFS($G$2:$G$48,$H$2:$H$48,$H13-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1205,7 +1276,7 @@
         <v/>
       </c>
       <c r="J14">
-        <f>IF($H14&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H14-4),"")</f>
+        <f>IF($H14&gt;=5,$G14-SUMIFS($G$2:$G$48,$H$2:$H$48,$H14-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1241,7 +1312,7 @@
         <v/>
       </c>
       <c r="J15">
-        <f>IF($H15&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H15-4),"")</f>
+        <f>IF($H15&gt;=5,$G15-SUMIFS($G$2:$G$48,$H$2:$H$48,$H15-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1277,7 +1348,7 @@
         <v/>
       </c>
       <c r="J16">
-        <f>IF($H16&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H16-4),"")</f>
+        <f>IF($H16&gt;=5,$G16-SUMIFS($G$2:$G$48,$H$2:$H$48,$H16-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1313,7 +1384,7 @@
         <v/>
       </c>
       <c r="J17">
-        <f>IF($H17&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H17-4),"")</f>
+        <f>IF($H17&gt;=5,$G17-SUMIFS($G$2:$G$48,$H$2:$H$48,$H17-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1349,7 +1420,7 @@
         <v/>
       </c>
       <c r="J18">
-        <f>IF($H18&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H18-4),"")</f>
+        <f>IF($H18&gt;=5,$G18-SUMIFS($G$2:$G$48,$H$2:$H$48,$H18-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1385,7 +1456,7 @@
         <v/>
       </c>
       <c r="J19">
-        <f>IF($H19&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H19-4),"")</f>
+        <f>IF($H19&gt;=5,$G19-SUMIFS($G$2:$G$48,$H$2:$H$48,$H19-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1421,7 +1492,7 @@
         <v/>
       </c>
       <c r="J20">
-        <f>IF($H20&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H20-4),"")</f>
+        <f>IF($H20&gt;=5,$G20-SUMIFS($G$2:$G$48,$H$2:$H$48,$H20-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1457,7 +1528,7 @@
         <v/>
       </c>
       <c r="J21">
-        <f>IF($H21&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H21-4),"")</f>
+        <f>IF($H21&gt;=5,$G21-SUMIFS($G$2:$G$48,$H$2:$H$48,$H21-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1493,7 +1564,7 @@
         <v/>
       </c>
       <c r="J22">
-        <f>IF($H22&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H22-4),"")</f>
+        <f>IF($H22&gt;=5,$G22-SUMIFS($G$2:$G$48,$H$2:$H$48,$H22-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1529,7 +1600,7 @@
         <v/>
       </c>
       <c r="J23">
-        <f>IF($H23&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H23-4),"")</f>
+        <f>IF($H23&gt;=5,$G23-SUMIFS($G$2:$G$48,$H$2:$H$48,$H23-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1565,7 +1636,7 @@
         <v/>
       </c>
       <c r="J24">
-        <f>IF($H24&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H24-4),"")</f>
+        <f>IF($H24&gt;=5,$G24-SUMIFS($G$2:$G$48,$H$2:$H$48,$H24-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1601,7 +1672,7 @@
         <v/>
       </c>
       <c r="J25">
-        <f>IF($H25&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H25-4),"")</f>
+        <f>IF($H25&gt;=5,$G25-SUMIFS($G$2:$G$48,$H$2:$H$48,$H25-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1637,7 +1708,7 @@
         <v/>
       </c>
       <c r="J26">
-        <f>IF($H26&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H26-4),"")</f>
+        <f>IF($H26&gt;=5,$G26-SUMIFS($G$2:$G$48,$H$2:$H$48,$H26-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1673,7 +1744,7 @@
         <v/>
       </c>
       <c r="J27">
-        <f>IF($H27&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H27-4),"")</f>
+        <f>IF($H27&gt;=5,$G27-SUMIFS($G$2:$G$48,$H$2:$H$48,$H27-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1709,7 +1780,7 @@
         <v/>
       </c>
       <c r="J28">
-        <f>IF($H28&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H28-4),"")</f>
+        <f>IF($H28&gt;=5,$G28-SUMIFS($G$2:$G$48,$H$2:$H$48,$H28-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1745,7 +1816,7 @@
         <v/>
       </c>
       <c r="J29">
-        <f>IF($H29&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H29-4),"")</f>
+        <f>IF($H29&gt;=5,$G29-SUMIFS($G$2:$G$48,$H$2:$H$48,$H29-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1781,7 +1852,7 @@
         <v/>
       </c>
       <c r="J30">
-        <f>IF($H30&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H30-4),"")</f>
+        <f>IF($H30&gt;=5,$G30-SUMIFS($G$2:$G$48,$H$2:$H$48,$H30-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1817,7 +1888,7 @@
         <v/>
       </c>
       <c r="J31">
-        <f>IF($H31&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H31-4),"")</f>
+        <f>IF($H31&gt;=5,$G31-SUMIFS($G$2:$G$48,$H$2:$H$48,$H31-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1853,7 +1924,7 @@
         <v/>
       </c>
       <c r="J32">
-        <f>IF($H32&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H32-4),"")</f>
+        <f>IF($H32&gt;=5,$G32-SUMIFS($G$2:$G$48,$H$2:$H$48,$H32-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1889,7 +1960,7 @@
         <v/>
       </c>
       <c r="J33">
-        <f>IF($H33&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H33-4),"")</f>
+        <f>IF($H33&gt;=5,$G33-SUMIFS($G$2:$G$48,$H$2:$H$48,$H33-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1925,7 +1996,7 @@
         <v/>
       </c>
       <c r="J34">
-        <f>IF($H34&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H34-4),"")</f>
+        <f>IF($H34&gt;=5,$G34-SUMIFS($G$2:$G$48,$H$2:$H$48,$H34-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1961,7 +2032,7 @@
         <v/>
       </c>
       <c r="J35">
-        <f>IF($H35&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H35-4),"")</f>
+        <f>IF($H35&gt;=5,$G35-SUMIFS($G$2:$G$48,$H$2:$H$48,$H35-4),"")</f>
         <v/>
       </c>
     </row>
@@ -1997,7 +2068,7 @@
         <v/>
       </c>
       <c r="J36">
-        <f>IF($H36&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H36-4),"")</f>
+        <f>IF($H36&gt;=5,$G36-SUMIFS($G$2:$G$48,$H$2:$H$48,$H36-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2033,7 +2104,7 @@
         <v/>
       </c>
       <c r="J37">
-        <f>IF($H37&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H37-4),"")</f>
+        <f>IF($H37&gt;=5,$G37-SUMIFS($G$2:$G$48,$H$2:$H$48,$H37-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2069,7 +2140,7 @@
         <v/>
       </c>
       <c r="J38">
-        <f>IF($H38&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H38-4),"")</f>
+        <f>IF($H38&gt;=5,$G38-SUMIFS($G$2:$G$48,$H$2:$H$48,$H38-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2105,7 +2176,7 @@
         <v/>
       </c>
       <c r="J39">
-        <f>IF($H39&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H39-4),"")</f>
+        <f>IF($H39&gt;=5,$G39-SUMIFS($G$2:$G$48,$H$2:$H$48,$H39-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2141,7 +2212,7 @@
         <v/>
       </c>
       <c r="J40">
-        <f>IF($H40&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H40-4),"")</f>
+        <f>IF($H40&gt;=5,$G40-SUMIFS($G$2:$G$48,$H$2:$H$48,$H40-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2177,7 +2248,7 @@
         <v/>
       </c>
       <c r="J41">
-        <f>IF($H41&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H41-4),"")</f>
+        <f>IF($H41&gt;=5,$G41-SUMIFS($G$2:$G$48,$H$2:$H$48,$H41-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2213,7 +2284,7 @@
         <v/>
       </c>
       <c r="J42">
-        <f>IF($H42&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H42-4),"")</f>
+        <f>IF($H42&gt;=5,$G42-SUMIFS($G$2:$G$48,$H$2:$H$48,$H42-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2249,7 +2320,7 @@
         <v/>
       </c>
       <c r="J43">
-        <f>IF($H43&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H43-4),"")</f>
+        <f>IF($H43&gt;=5,$G43-SUMIFS($G$2:$G$48,$H$2:$H$48,$H43-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2285,7 +2356,7 @@
         <v/>
       </c>
       <c r="J44">
-        <f>IF($H44&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H44-4),"")</f>
+        <f>IF($H44&gt;=5,$G44-SUMIFS($G$2:$G$48,$H$2:$H$48,$H44-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2321,7 +2392,7 @@
         <v/>
       </c>
       <c r="J45">
-        <f>IF($H45&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H45-4),"")</f>
+        <f>IF($H45&gt;=5,$G45-SUMIFS($G$2:$G$48,$H$2:$H$48,$H45-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2357,7 +2428,7 @@
         <v/>
       </c>
       <c r="J46">
-        <f>IF($H46&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H46-4),"")</f>
+        <f>IF($H46&gt;=5,$G46-SUMIFS($G$2:$G$48,$H$2:$H$48,$H46-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2393,7 +2464,7 @@
         <v/>
       </c>
       <c r="J47">
-        <f>IF($H47&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H47-4),"")</f>
+        <f>IF($H47&gt;=5,$G47-SUMIFS($G$2:$G$48,$H$2:$H$48,$H47-4),"")</f>
         <v/>
       </c>
     </row>
@@ -2429,12 +2500,17 @@
         <v/>
       </c>
       <c r="J48">
-        <f>IF($H48&gt;=5,SUMIFS($G$2:$G$48,$H$2:$H$48,$H48-4),"")</f>
+        <f>IF($H48&gt;=5,$G48-SUMIFS($G$2:$G$48,$H$2:$H$48,$H48-4),"")</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -2442,9 +2518,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2458,7 +2534,7 @@
     <col width="27" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Year</t>
@@ -2507,7 +2583,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="B2" s="11">
         <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A2)</f>
@@ -2521,9 +2597,7 @@
         <f>B2/C2*100</f>
         <v/>
       </c>
-      <c r="E2" s="11" t="n">
-        <v>4.9</v>
-      </c>
+      <c r="E2" s="11" t="n"/>
       <c r="F2" s="13" t="n"/>
       <c r="G2" s="13" t="n"/>
       <c r="H2" s="13" t="n"/>
@@ -2531,7 +2605,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="B3" s="11">
         <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A3)</f>
@@ -2546,7 +2620,7 @@
         <v/>
       </c>
       <c r="E3" s="11" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="F3" s="13">
         <f>B3-B2</f>
@@ -2567,7 +2641,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="B4" s="11">
         <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A4)</f>
@@ -2582,7 +2656,7 @@
         <v/>
       </c>
       <c r="E4" s="11" t="n">
-        <v>6</v>
+        <v>4.7</v>
       </c>
       <c r="F4" s="13">
         <f>B4-B3</f>
@@ -2603,7 +2677,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="B5" s="11">
         <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A5)</f>
@@ -2618,7 +2692,7 @@
         <v/>
       </c>
       <c r="E5" s="11" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="F5" s="13">
         <f>B5-B4</f>
@@ -2639,7 +2713,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B6" s="11">
         <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A6)</f>
@@ -2654,7 +2728,7 @@
         <v/>
       </c>
       <c r="E6" s="11" t="n">
-        <v>7.1</v>
+        <v>5.8</v>
       </c>
       <c r="F6" s="13">
         <f>B6-B5</f>
@@ -2675,7 +2749,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B7" s="11">
         <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A7)</f>
@@ -2690,7 +2764,7 @@
         <v/>
       </c>
       <c r="E7" s="11" t="n">
-        <v>4.5</v>
+        <v>7.1</v>
       </c>
       <c r="F7" s="13">
         <f>B7-B6</f>
@@ -2711,7 +2785,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B8" s="11">
         <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A8)</f>
@@ -2726,7 +2800,7 @@
         <v/>
       </c>
       <c r="E8" s="11" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F8" s="13">
         <f>B8-B7</f>
@@ -2747,7 +2821,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B9" s="11">
         <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A9)</f>
@@ -2762,7 +2836,7 @@
         <v/>
       </c>
       <c r="E9" s="11" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="F9" s="13">
         <f>B9-B8</f>
@@ -2783,7 +2857,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B10" s="11">
         <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A10)</f>
@@ -2798,7 +2872,7 @@
         <v/>
       </c>
       <c r="E10" s="11" t="n">
-        <v>5.4</v>
+        <v>4</v>
       </c>
       <c r="F10" s="13">
         <f>B10-B9</f>
@@ -2819,7 +2893,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B11" s="11">
         <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A11)</f>
@@ -2834,7 +2908,7 @@
         <v/>
       </c>
       <c r="E11" s="11" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="F11" s="13">
         <f>B11-B10</f>
@@ -2853,21 +2927,66 @@
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B12" s="11">
+        <f>SUMIFS(Quarterly!$F$2:$F$48,Quarterly!$B$2:$B$48,$A12)</f>
+        <v/>
+      </c>
+      <c r="C12" s="11">
+        <f>AVERAGEIFS(Quarterly!$E$2:$E$48,Quarterly!$B$2:$B$48,$A12)</f>
+        <v/>
+      </c>
+      <c r="D12" s="12">
+        <f>B12/C12*100</f>
+        <v/>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F12" s="13">
+        <f>B12-B11</f>
+        <v/>
+      </c>
+      <c r="G12" s="13">
+        <f>(C12-C11)*(D11+D12)/200</f>
+        <v/>
+      </c>
+      <c r="H12" s="13">
+        <f>(D12-D11)/100*(C11+C12)/2</f>
+        <v/>
+      </c>
+      <c r="I12" s="14">
+        <f>IF(F12="","",ROUND(F12-G12-H12,6))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Live formulas from the Quarterly sheet (SUMIFS / AVERAGEIFS) — the same midpoint split as outputs/yearly_bridge.csv.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Column E (published rate) is pasted from the MAS annual file; volume = Δrollover × avg rate · rate = Δrate × avg rollover.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I12"/>
+  <mergeCells count="2">
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A14:I14"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: validate quarter headers and preserve workbook provenance
Refs #9
</commit_message>
<xml_diff>
--- a/outputs/quick_check.xlsx
+++ b/outputs/quick_check.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Annual bridge" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quick check'!$A$1:$B$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quick check'!$A$1:$B$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Quarterly'!$A$1:$J$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Quarterly'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Quarterly'!$A$1:$J$48</definedName>
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -693,26 +693,33 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Charge-off rate is as published: bad debts written off ÷ average rollover balance, annualised.</t>
+          <t>Published rate: source percentage; publisher averaging/write-off treatment unverified.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Formula-only, no macros. XLOOKUP needs Excel 2021+/365; older readers can swap it for INDEX/MATCH.</t>
+          <t>Proxy = annual write-offs / mean quarter-end rollover; not a verified publisher denominator.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>Formula-only, no macros. XLOOKUP needs Excel 2021+/365; older readers can swap it for INDEX/MATCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>Numbers reproduce outputs/yearly_bridge.csv and the README headline for the same pull.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A16:B16"/>
@@ -727,6 +734,7 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A27:B27"/>
     <mergeCell ref="A22:B22"/>
   </mergeCells>
   <dataValidations count="1">

</xml_diff>

<commit_message>
fix: validate quarter headers and preserve workbook provenance (#10)
Refs #9

Co-authored-by: Muhammad Faiz Saifulnizam <240133439+faizsaifulnizam@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/quick_check.xlsx
+++ b/outputs/quick_check.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Annual bridge" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quick check'!$A$1:$B$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quick check'!$A$1:$B$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Quarterly'!$A$1:$J$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Quarterly'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Quarterly'!$A$1:$J$48</definedName>
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -693,26 +693,33 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Charge-off rate is as published: bad debts written off ÷ average rollover balance, annualised.</t>
+          <t>Published rate: source percentage; publisher averaging/write-off treatment unverified.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Formula-only, no macros. XLOOKUP needs Excel 2021+/365; older readers can swap it for INDEX/MATCH.</t>
+          <t>Proxy = annual write-offs / mean quarter-end rollover; not a verified publisher denominator.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>Formula-only, no macros. XLOOKUP needs Excel 2021+/365; older readers can swap it for INDEX/MATCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>Numbers reproduce outputs/yearly_bridge.csv and the README headline for the same pull.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A16:B16"/>
@@ -727,6 +734,7 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A27:B27"/>
     <mergeCell ref="A22:B22"/>
   </mergeCells>
   <dataValidations count="1">

</xml_diff>